<commit_message>
Add 7 new IMG-route and comparison posts for uncovered keywords
Covers the highest-priority terms from UKMLA_SEO_Keyword_Research.xlsx's
"All Keywords (Final)" backlog (India/Pakistan/Nigeria IMG routes, UKMLA
vs USMLE, UKMLA vs NEET PG, question bank/mock test guide, IMG fees),
clustered to avoid keyword cannibalization. Each post is 5,000+ words
with real featured images, natural internal linking, and GMC sourcing.
Regenerates all three tracking workbooks and the linking cluster rules.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UKMLA_Internal_Linking_Map.xlsx
+++ b/UKMLA_Internal_Linking_Map.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internal Linking Map'!$A$1:$I$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Internal Linking Map'!$A$1:$I$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -526,14 +526,14 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; MLA Content Map: The Blueprint Behind Every UKMLA Question; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Social Determinants of Health in the UKMLA: Person-Centred Care; Time Management in the UKMLA AKT: Strategies That Work; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; How to Become a Doctor in the UK from India: The Complete UKMLA Route; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; MLA Content Map: The Blueprint Behind Every UKMLA Question; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Social Determinants of Health in the UKMLA: Person-Centred Care; Time Management in the UKMLA AKT: Strategies That Work; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs PLAB: What Is the Difference?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr"/>
@@ -561,14 +561,14 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; How to Become a Doctor in the UK from India: The Complete UKMLA Route; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr"/>
@@ -596,14 +596,14 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Emergency Medicine and Acute Presentations in the UKMLA; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; Gastroenterology and Hepatology in the UKMLA AKT; Good Medical Practice and the UKMLA: What the GMC Expects; How to Read an AKT Stem: Avoiding Common Traps; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; Mental Health Presentations in the UKMLA: What to Revise; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; NICE Guidelines and the AKT: What You Actually Need to Know; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Safeguarding Adults and Children: A UKMLA Revision Guide; Social Determinants of Health in the UKMLA: Person-Centred Care; Three Months to the UKMLA AKT: A Final Preparation Countdown; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Emergency Medicine and Acute Presentations in the UKMLA; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; Gastroenterology and Hepatology in the UKMLA AKT; Good Medical Practice and the UKMLA: What the GMC Expects; How to Become a Doctor in the UK from India: The Complete UKMLA Route; How to Read an AKT Stem: Avoiding Common Traps; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; Mental Health Presentations in the UKMLA: What to Revise; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; NICE Guidelines and the AKT: What You Actually Need to Know; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Safeguarding Adults and Children: A UKMLA Revision Guide; Social Determinants of Health in the UKMLA: Person-Centred Care; Three Months to the UKMLA AKT: A Final Preparation Countdown; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs PLAB: What Is the Difference?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr"/>
@@ -631,14 +631,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Understanding the Foundation Programme: What Awaits After the UKMLA; Good Medical Practice and the UKMLA: What the GMC Expects; Mental Health Presentations in the UKMLA: What to Revise; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Psychiatry Communication Stations: Handling Difficult Conversations; Respiratory Medicine for the UKMLA: What to Focus On; Safeguarding Adults and Children: A UKMLA Revision Guide; Three Months to the UKMLA AKT: A Final Preparation Countdown; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Understanding the Foundation Programme: What Awaits After the UKMLA; Good Medical Practice and the UKMLA: What the GMC Expects; How to Become a Doctor in the UK from India: The Complete UKMLA Route; Mental Health Presentations in the UKMLA: What to Revise; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Psychiatry Communication Stations: Handling Difficult Conversations; Respiratory Medicine for the UKMLA: What to Focus On; Safeguarding Adults and Children: A UKMLA Revision Guide; Three Months to the UKMLA AKT: A Final Preparation Countdown; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs PLAB: What Is the Difference?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
@@ -666,14 +666,14 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>How to Become a Doctor in the UK from India: The Complete UKMLA Route; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs PLAB: What Is the Difference?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr"/>
@@ -701,14 +701,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Understanding the Foundation Programme: What Awaits After the UKMLA; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
+          <t>Understanding the Foundation Programme: What Awaits After the UKMLA; How to Become a Doctor in the UK from India: The Complete UKMLA Route; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr"/>
@@ -736,14 +736,14 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>What Is an Angoff Standard Setting and Why Does It Matter?; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>What Is an Angoff Standard Setting and Why Does It Matter?; How to Become a Doctor in the UK from India: The Complete UKMLA Route; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr"/>
@@ -771,14 +771,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Emergency Medicine and Acute Presentations in the UKMLA; Understanding the Foundation Programme: What Awaits After the UKMLA; Gastroenterology and Hepatology in the UKMLA AKT; Good Medical Practice and the UKMLA: What the GMC Expects; Group Study vs Solo Study for the UKMLA: What Works Best?; How to Read an AKT Stem: Avoiding Common Traps; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Neurology in the UKMLA: High-Yield Topics and Revision Tips; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Safeguarding Adults and Children: A UKMLA Revision Guide; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Emergency Medicine and Acute Presentations in the UKMLA; Understanding the Foundation Programme: What Awaits After the UKMLA; Gastroenterology and Hepatology in the UKMLA AKT; Good Medical Practice and the UKMLA: What the GMC Expects; Group Study vs Solo Study for the UKMLA: What Works Best?; How to Read an AKT Stem: Avoiding Common Traps; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Neurology in the UKMLA: High-Yield Topics and Revision Tips; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Safeguarding Adults and Children: A UKMLA Revision Guide; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr"/>
@@ -806,14 +806,14 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; PLAB 2 Preparation: How to Excel in the Clinical Assessment; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; How to Become a Doctor in the UK from India: The Complete UKMLA Route; PLAB 2 Preparation: How to Excel in the Clinical Assessment; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs PLAB: What Is the Difference?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr"/>
@@ -841,14 +841,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>What Is an Angoff Standard Setting and Why Does It Matter?; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Understanding the Foundation Programme: What Awaits After the UKMLA; The Role of Mock Exams in UKMLA Preparation; PLAB 2 Preparation: How to Excel in the Clinical Assessment; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>What Is an Angoff Standard Setting and Why Does It Matter?; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Understanding the Foundation Programme: What Awaits After the UKMLA; The Role of Mock Exams in UKMLA Preparation; PLAB 2 Preparation: How to Excel in the Clinical Assessment; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs PLAB: What Is the Difference?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr"/>
@@ -876,14 +876,14 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Understanding the Foundation Programme: What Awaits After the UKMLA; Gastroenterology and Hepatology in the UKMLA AKT; Good Medical Practice and the UKMLA: What the GMC Expects; Group Study vs Solo Study for the UKMLA: What Works Best?; How to Read an AKT Stem: Avoiding Common Traps; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Psychiatry Communication Stations: Handling Difficult Conversations; Respiratory Medicine for the UKMLA: What to Focus On; Safeguarding Adults and Children: A UKMLA Revision Guide; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Understanding the Foundation Programme: What Awaits After the UKMLA; Gastroenterology and Hepatology in the UKMLA AKT; Good Medical Practice and the UKMLA: What the GMC Expects; Group Study vs Solo Study for the UKMLA: What Works Best?; How to Read an AKT Stem: Avoiding Common Traps; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Psychiatry Communication Stations: Handling Difficult Conversations; Respiratory Medicine for the UKMLA: What to Focus On; Safeguarding Adults and Children: A UKMLA Revision Guide; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs PLAB: What Is the Difference?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr"/>
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; MLA Content Map: The Blueprint Behind Every UKMLA Question; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; How to Become a Doctor in the UK from India: The Complete UKMLA Route; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; MLA Content Map: The Blueprint Behind Every UKMLA Question; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs PLAB: What Is the Difference?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr"/>
@@ -946,14 +946,14 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Clinical Examination Stations in the CPSA: A Practical Guide; Emergency Medicine and Acute Presentations in the UKMLA; Understanding the Foundation Programme: What Awaits After the UKMLA; Good Medical Practice and the UKMLA: What the GMC Expects; How to Read an AKT Stem: Avoiding Common Traps; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA for Graduate-Entry Medical Students: What Is Different?; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>Clinical Examination Stations in the CPSA: A Practical Guide; Emergency Medicine and Acute Presentations in the UKMLA; Understanding the Foundation Programme: What Awaits After the UKMLA; Good Medical Practice and the UKMLA: What the GMC Expects; How to Read an AKT Stem: Avoiding Common Traps; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA for Graduate-Entry Medical Students: What Is Different?; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs PLAB: What Is the Difference?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr"/>
@@ -981,14 +981,14 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>16</v>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>UKMLA Results: How to Interpret Your Feedback Report; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1024,14 +1024,14 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>10</v>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Clinical Examination Stations in the CPSA: A Practical Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Good Medical Practice and the UKMLA: What the GMC Expects; The Role of Mock Exams in UKMLA Preparation; Radiology and Imaging Interpretation in the AKT; Safeguarding Adults and Children: A UKMLA Revision Guide; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Results: How to Interpret Your Feedback Report</t>
+          <t>Clinical Examination Stations in the CPSA: A Practical Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Good Medical Practice and the UKMLA: What the GMC Expects; The Role of Mock Exams in UKMLA Preparation; Radiology and Imaging Interpretation in the AKT; Safeguarding Adults and Children: A UKMLA Revision Guide; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1067,14 +1067,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>9</v>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Clinical Examination Stations in the CPSA: A Practical Guide; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Emergency Medicine and Acute Presentations in the UKMLA; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Gastroenterology and Hepatology in the UKMLA AKT; Group Study vs Solo Study for the UKMLA: What Works Best?; How to Read an AKT Stem: Avoiding Common Traps; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Nephrology in the UKMLA: AKI, CKD, and Electrolyte Disorders; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Psychiatry Communication Stations: Handling Difficult Conversations; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Social Determinants of Health in the UKMLA: Person-Centred Care; Three Months to the UKMLA AKT: A Final Preparation Countdown; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work</t>
+          <t>Clinical Examination Stations in the CPSA: A Practical Guide; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Emergency Medicine and Acute Presentations in the UKMLA; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Gastroenterology and Hepatology in the UKMLA AKT; Group Study vs Solo Study for the UKMLA: What Works Best?; How to Read an AKT Stem: Avoiding Common Traps; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Nephrology in the UKMLA: AKI, CKD, and Electrolyte Disorders; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Psychiatry Communication Stations: Handling Difficult Conversations; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Social Determinants of Health in the UKMLA: Person-Centred Care; Three Months to the UKMLA AKT: A Final Preparation Countdown; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1110,14 +1110,14 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>13</v>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Understanding the Foundation Programme: What Awaits After the UKMLA; Group Study vs Solo Study for the UKMLA: What Works Best?; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; PLAB 2 Preparation: How to Excel in the Clinical Assessment; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Understanding the Foundation Programme: What Awaits After the UKMLA; Group Study vs Solo Study for the UKMLA: What Works Best?; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; PLAB 2 Preparation: How to Excel in the Clinical Assessment; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -1153,14 +1153,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>9</v>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA AKT: Format, Question Types, and How to Prepare</t>
+          <t>Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1282,14 +1282,14 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>12</v>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Understanding the Foundation Programme: What Awaits After the UKMLA; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; Paediatrics in the AKT and CPSA: A Focused Revision Guide</t>
+          <t>Understanding the Foundation Programme: What Awaits After the UKMLA; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; Paediatrics in the AKT and CPSA: A Focused Revision Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -1325,14 +1325,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>8</v>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Emergency Medicine and Acute Presentations in the UKMLA; Gastroenterology and Hepatology in the UKMLA AKT; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; Nephrology in the UKMLA: AKI, CKD, and Electrolyte Disorders; Neurology in the UKMLA: High-Yield Topics and Revision Tips; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Social Determinants of Health in the UKMLA: Person-Centred Care; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; Time Management in the UKMLA AKT: Strategies That Work; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
+          <t>Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Emergency Medicine and Acute Presentations in the UKMLA; Gastroenterology and Hepatology in the UKMLA AKT; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; Nephrology in the UKMLA: AKI, CKD, and Electrolyte Disorders; Neurology in the UKMLA: High-Yield Topics and Revision Tips; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Social Determinants of Health in the UKMLA: Person-Centred Care; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; Time Management in the UKMLA AKT: Strategies That Work; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1368,14 +1368,14 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>20</v>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>What Is an Angoff Standard Setting and Why Does It Matter?; MLA Content Map: The Blueprint Behind Every UKMLA Question; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>What Is an Angoff Standard Setting and Why Does It Matter?; MLA Content Map: The Blueprint Behind Every UKMLA Question; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs PLAB: What Is the Difference?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -1561,12 +1561,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>How to Read an AKT Stem: Avoiding Common Traps</t>
+          <t>How to Become a Doctor in the UK from India: The Complete UKMLA Route</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>/news#how-to-read-akt-stem</t>
+          <t>/news#how-to-become-a-doctor-in-uk-from-india</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1575,41 +1575,41 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Group Study vs Solo Study for the UKMLA: What Works Best?; The Role of Mock Exams in UKMLA Preparation; Three Months to the UKMLA AKT: A Final Preparation Countdown; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs PLAB: What Is the Difference?</t>
+          <t>UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>AKT Exam Pattern; Preparation; MLA Content Map / Syllabus; What Is the UKMLA?; Cardiology High-Yield Topics for the UKMLA AKT; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; The Role of Mock Exams in UKMLA Preparation; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Safeguarding Adults and Children: A UKMLA Revision Guide; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; How UK Medical Schools Implement the UKMLA: An Overview</t>
+          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; CPSA Exam Pattern; Fees; Key Dates; Official Resources; Registration Guide; UKMLA vs PLAB; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; PLAB 2 Preparation: How to Excel in the Clinical Assessment; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Exam Format</t>
+          <t>IMG Country Routes &amp; Global Comparisons</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>AKT Exam Pattern</t>
+          <t>Eligibility</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>How to Register for PLAB 1: A Step-by-Step Guide for IMGs</t>
+          <t>How to Read an AKT Stem: Avoiding Common Traps</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>/news#how-to-register-plab-1</t>
+          <t>/news#how-to-read-akt-stem</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1618,41 +1618,41 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA vs PLAB: What Is the Difference?</t>
+          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Group Study vs Solo Study for the UKMLA: What Works Best?; The Role of Mock Exams in UKMLA Preparation; Three Months to the UKMLA AKT: A Final Preparation Countdown; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs PLAB: What Is the Difference?</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; Key Dates; Official Resources; Preparation; MLA Content Map / Syllabus; UKMLA vs PLAB; The Role of Mock Exams in UKMLA Preparation; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Key Dates and Sitting Schedule: What to Know</t>
+          <t>AKT Exam Pattern; Preparation; MLA Content Map / Syllabus; What Is the UKMLA?; Cardiology High-Yield Topics for the UKMLA AKT; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; The Role of Mock Exams in UKMLA Preparation; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Safeguarding Adults and Children: A UKMLA Revision Guide; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; How UK Medical Schools Implement the UKMLA: An Overview</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Registration &amp; Eligibility</t>
+          <t>Exam Format</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Registration Guide</t>
+          <t>AKT Exam Pattern</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More</t>
+          <t>How to Register for PLAB 1: A Step-by-Step Guide for IMGs</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>/news#infection-microbiology-ukmla-revision</t>
+          <t>/news#how-to-register-plab-1</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1661,41 +1661,41 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Emergency Medicine and Acute Presentations in the UKMLA; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; Gastroenterology and Hepatology in the UKMLA AKT; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; How to Read an AKT Stem: Avoiding Common Traps; MLA Content Map: The Blueprint Behind Every UKMLA Question; Nephrology in the UKMLA: AKI, CKD, and Electrolyte Disorders; Neurology in the UKMLA: High-Yield Topics and Revision Tips; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Radiology and Imaging Interpretation in the AKT; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Safeguarding Adults and Children: A UKMLA Revision Guide; Social Determinants of Health in the UKMLA: Person-Centred Care; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA for Graduate-Entry Medical Students: What Is Different?</t>
+          <t>How to Become a Doctor in the UK from India: The Complete UKMLA Route; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA vs PLAB: What Is the Difference?</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Preparation; Gastroenterology and Hepatology in the UKMLA AKT; Mental Health Presentations in the UKMLA: What to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know</t>
+          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; Key Dates; Official Resources; Preparation; MLA Content Map / Syllabus; UKMLA vs PLAB; The Role of Mock Exams in UKMLA Preparation; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Key Dates and Sitting Schedule: What to Know</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Clinical Systems Revision</t>
+          <t>Registration &amp; Eligibility</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>MLA Content Map / Syllabus</t>
+          <t>Registration Guide</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Mental Health Presentations in the UKMLA: What to Revise</t>
+          <t>Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>/news#mental-health-ukmla-revision</t>
+          <t>/news#infection-microbiology-ukmla-revision</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1704,19 +1704,19 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Good Medical Practice and the UKMLA: What the GMC Expects; How to Read an AKT Stem: Avoiding Common Traps; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Psychiatry Communication Stations: Handling Difficult Conversations; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Safeguarding Adults and Children: A UKMLA Revision Guide; Social Determinants of Health in the UKMLA: Person-Centred Care; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
+          <t>Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Emergency Medicine and Acute Presentations in the UKMLA; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; Gastroenterology and Hepatology in the UKMLA AKT; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; How to Read an AKT Stem: Avoiding Common Traps; MLA Content Map: The Blueprint Behind Every UKMLA Question; Nephrology in the UKMLA: AKI, CKD, and Electrolyte Disorders; Neurology in the UKMLA: High-Yield Topics and Revision Tips; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Radiology and Imaging Interpretation in the AKT; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Safeguarding Adults and Children: A UKMLA Revision Guide; Social Determinants of Health in the UKMLA: Person-Centred Care; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>AKT Exam Pattern; CPSA Exam Pattern; Preparation; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; MLA Content Map: The Blueprint Behind Every UKMLA Question; NICE Guidelines and the AKT: What You Actually Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Psychiatry Communication Stations: Handling Difficult Conversations; Three Months to the UKMLA AKT: A Final Preparation Countdown; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA CPSA: What the Clinical Exam Really Tests</t>
+          <t>Preparation; Gastroenterology and Hepatology in the UKMLA AKT; Mental Health Presentations in the UKMLA: What to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1733,12 +1733,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>MLA Content Map: The Blueprint Behind Every UKMLA Question</t>
+          <t>Mental Health Presentations in the UKMLA: What to Revise</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>/news#mla-content-map-explained</t>
+          <t>/news#mental-health-ukmla-revision</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1747,24 +1747,24 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Mental Health Presentations in the UKMLA: What to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide</t>
+          <t>Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Good Medical Practice and the UKMLA: What the GMC Expects; How to Read an AKT Stem: Avoiding Common Traps; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Psychiatry Communication Stations: Handling Difficult Conversations; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Safeguarding Adults and Children: A UKMLA Revision Guide; Social Determinants of Health in the UKMLA: Person-Centred Care; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Appeals and Resits; AKT Exam Pattern; CPSA Exam Pattern; Official Resources; Preparation; MLA Content Map / Syllabus; UKMLA vs PLAB; What Is the UKMLA?; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Understanding the Foundation Programme: What Awaits After the UKMLA; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Safeguarding Adults and Children: A UKMLA Revision Guide; Social Determinants of Health in the UKMLA: Person-Centred Care; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA vs PLAB: What Is the Difference?</t>
+          <t>AKT Exam Pattern; CPSA Exam Pattern; Preparation; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; MLA Content Map: The Blueprint Behind Every UKMLA Question; NICE Guidelines and the AKT: What You Actually Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Psychiatry Communication Stations: Handling Difficult Conversations; Three Months to the UKMLA AKT: A Final Preparation Countdown; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA CPSA: What the Clinical Exam Really Tests</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Core UKMLA Overview</t>
+          <t>Clinical Systems Revision</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -1776,12 +1776,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>The Role of Mock Exams in UKMLA Preparation</t>
+          <t>MLA Content Map: The Blueprint Behind Every UKMLA Question</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>/news#mock-exams-ukmla-preparation</t>
+          <t>/news#mla-content-map-explained</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1790,41 +1790,41 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Clinical Examination Stations in the CPSA: A Practical Guide; Group Study vs Solo Study for the UKMLA: What Works Best?; How to Read an AKT Stem: Avoiding Common Traps; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Time Management in the UKMLA AKT: Strategies That Work; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA vs PLAB: What Is the Difference?</t>
+          <t>Mental Health Presentations in the UKMLA: What to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>AKT Exam Pattern; CPSA Exam Pattern; Official Resources; Preparation; Results and Scoring; MLA Content Map / Syllabus; What Is the UKMLA?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Gastroenterology and Hepatology in the UKMLA AKT; How to Read an AKT Stem: Avoiding Common Traps; Mental Health Presentations in the UKMLA: What to Revise; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Psychiatry Communication Stations: Handling Difficult Conversations; Respiratory Medicine for the UKMLA: What to Focus On; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare</t>
+          <t>Appeals and Resits; AKT Exam Pattern; CPSA Exam Pattern; Official Resources; Preparation; MLA Content Map / Syllabus; UKMLA vs PLAB; What Is the UKMLA?; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Understanding the Foundation Programme: What Awaits After the UKMLA; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Safeguarding Adults and Children: A UKMLA Revision Guide; Social Determinants of Health in the UKMLA: Person-Centred Care; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA vs PLAB: What Is the Difference?</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Exam Preparation</t>
+          <t>Core UKMLA Overview</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Preparation</t>
+          <t>MLA Content Map / Syllabus</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Nephrology in the UKMLA: AKI, CKD, and Electrolyte Disorders</t>
+          <t>The Role of Mock Exams in UKMLA Preparation</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>/news#nephrology-ukmla-revision</t>
+          <t>/news#mock-exams-ukmla-preparation</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -1833,41 +1833,41 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>NICE Guidelines and the AKT: What You Actually Need to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown</t>
+          <t>Clinical Examination Stations in the CPSA: A Practical Guide; Group Study vs Solo Study for the UKMLA: What Works Best?; How to Read an AKT Stem: Avoiding Common Traps; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Time Management in the UKMLA AKT: Strategies That Work; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA vs PLAB: What Is the Difference?</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Cardiology High-Yield Topics for the UKMLA AKT; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know</t>
+          <t>AKT Exam Pattern; CPSA Exam Pattern; Official Resources; Preparation; Results and Scoring; MLA Content Map / Syllabus; What Is the UKMLA?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Gastroenterology and Hepatology in the UKMLA AKT; How to Read an AKT Stem: Avoiding Common Traps; Mental Health Presentations in the UKMLA: What to Revise; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Psychiatry Communication Stations: Handling Difficult Conversations; Respiratory Medicine for the UKMLA: What to Focus On; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Clinical Systems Revision</t>
+          <t>Exam Preparation</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>MLA Content Map / Syllabus</t>
+          <t>Preparation</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Neurology in the UKMLA: High-Yield Topics and Revision Tips</t>
+          <t>Nephrology in the UKMLA: AKI, CKD, and Electrolyte Disorders</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>/news#neurology-ukmla-revision</t>
+          <t>/news#nephrology-ukmla-revision</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1876,19 +1876,19 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Clinical Examination Stations in the CPSA: A Practical Guide; Emergency Medicine and Acute Presentations in the UKMLA; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Graduate-Entry Medical Students: What Is Different?; How to Write UKMLA Revision Notes That Actually Work</t>
+          <t>NICE Guidelines and the AKT: What You Actually Need to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Preparation; MLA Content Map / Syllabus; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; UKMLA CPSA: What the Clinical Exam Really Tests</t>
+          <t>Cardiology High-Yield Topics for the UKMLA AKT; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -1905,12 +1905,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>NICE Guidelines and the AKT: What You Actually Need to Know</t>
+          <t>Neurology in the UKMLA: High-Yield Topics and Revision Tips</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>/news#nice-guidelines-akt-revision</t>
+          <t>/news#neurology-ukmla-revision</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -1919,19 +1919,19 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Cardiology High-Yield Topics for the UKMLA AKT; ECG Interpretation for the UKMLA: The Findings You Must Recognise; How to Read an AKT Stem: Avoiding Common Traps; Mental Health Presentations in the UKMLA: What to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Safeguarding Adults and Children: A UKMLA Revision Guide; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide; How to Write UKMLA Revision Notes That Actually Work</t>
+          <t>Clinical Examination Stations in the CPSA: A Practical Guide; Emergency Medicine and Acute Presentations in the UKMLA; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Graduate-Entry Medical Students: What Is Different?; How to Write UKMLA Revision Notes That Actually Work</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>AKT Exam Pattern; Preparation; Cardiology High-Yield Topics for the UKMLA AKT; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; Nephrology in the UKMLA: AKI, CKD, and Electrolyte Disorders; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Respiratory Medicine for the UKMLA: What to Focus On</t>
+          <t>Preparation; MLA Content Map / Syllabus; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; UKMLA CPSA: What the Clinical Exam Really Tests</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -1948,12 +1948,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise</t>
+          <t>NICE Guidelines and the AKT: What You Actually Need to Know</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>/news#obstetrics-gynaecology-ukmla-revision</t>
+          <t>/news#nice-guidelines-akt-revision</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -1962,19 +1962,19 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Understanding the Foundation Programme: What Awaits After the UKMLA; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; How to Read an AKT Stem: Avoiding Common Traps; MLA Content Map: The Blueprint Behind Every UKMLA Question; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Radiology and Imaging Interpretation in the AKT; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Results: How to Interpret Your Feedback Report</t>
+          <t>Cardiology High-Yield Topics for the UKMLA AKT; ECG Interpretation for the UKMLA: The Findings You Must Recognise; How to Read an AKT Stem: Avoiding Common Traps; Mental Health Presentations in the UKMLA: What to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Safeguarding Adults and Children: A UKMLA Revision Guide; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide; How to Write UKMLA Revision Notes That Actually Work</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Preparation; MLA Content Map / Syllabus; Cardiology High-Yield Topics for the UKMLA AKT; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know</t>
+          <t>AKT Exam Pattern; Preparation; Cardiology High-Yield Topics for the UKMLA AKT; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; Nephrology in the UKMLA: AKI, CKD, and Electrolyte Disorders; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Respiratory Medicine for the UKMLA: What to Focus On</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -1991,12 +1991,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know</t>
+          <t>Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>/news#ophthalmology-ent-ukmla-revision</t>
+          <t>/news#obstetrics-gynaecology-ukmla-revision</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2005,19 +2005,19 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>11</v>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Palliative Care and End-of-Life Decisions in the UKMLA; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Safeguarding Adults and Children: A UKMLA Revision Guide; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA AKT: Format, Question Types, and How to Prepare</t>
+          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Understanding the Foundation Programme: What Awaits After the UKMLA; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; How to Read an AKT Stem: Avoiding Common Traps; MLA Content Map: The Blueprint Behind Every UKMLA Question; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Radiology and Imaging Interpretation in the AKT; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>AKT Exam Pattern; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Neurology in the UKMLA: High-Yield Topics and Revision Tips; NICE Guidelines and the AKT: What You Actually Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; How UK Medical Schools Implement the UKMLA: An Overview</t>
+          <t>Preparation; MLA Content Map / Syllabus; Cardiology High-Yield Topics for the UKMLA AKT; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2034,12 +2034,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Paediatrics in the AKT and CPSA: A Focused Revision Guide</t>
+          <t>Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>/news#paediatrics-ukmla-revision</t>
+          <t>/news#ophthalmology-ent-ukmla-revision</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2048,19 +2048,19 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Emergency Medicine and Acute Presentations in the UKMLA; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; Good Medical Practice and the UKMLA: What the GMC Expects; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; How to Read an AKT Stem: Avoiding Common Traps; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Safeguarding Adults and Children: A UKMLA Revision Guide; Social Determinants of Health in the UKMLA: Person-Centred Care; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Results: How to Interpret Your Feedback Report</t>
+          <t>Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Palliative Care and End-of-Life Decisions in the UKMLA; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Safeguarding Adults and Children: A UKMLA Revision Guide; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>CPSA Exam Pattern; Preparation; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Emergency Medicine and Acute Presentations in the UKMLA; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; MLA Content Map: The Blueprint Behind Every UKMLA Question; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Respiratory Medicine for the UKMLA: What to Focus On; Safeguarding Adults and Children: A UKMLA Revision Guide; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown</t>
+          <t>AKT Exam Pattern; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Neurology in the UKMLA: High-Yield Topics and Revision Tips; NICE Guidelines and the AKT: What You Actually Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; How UK Medical Schools Implement the UKMLA: An Overview</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2077,12 +2077,12 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Palliative Care and End-of-Life Decisions in the UKMLA</t>
+          <t>Paediatrics in the AKT and CPSA: A Focused Revision Guide</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>/news#palliative-care-ukmla-revision</t>
+          <t>/news#paediatrics-ukmla-revision</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2091,19 +2091,19 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA Results: How to Interpret Your Feedback Report</t>
+          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Emergency Medicine and Acute Presentations in the UKMLA; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; Good Medical Practice and the UKMLA: What the GMC Expects; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; How to Read an AKT Stem: Avoiding Common Traps; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Safeguarding Adults and Children: A UKMLA Revision Guide; Social Determinants of Health in the UKMLA: Person-Centred Care; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know</t>
+          <t>CPSA Exam Pattern; Preparation; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Emergency Medicine and Acute Presentations in the UKMLA; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; MLA Content Map: The Blueprint Behind Every UKMLA Question; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Respiratory Medicine for the UKMLA: What to Focus On; Safeguarding Adults and Children: A UKMLA Revision Guide; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2120,12 +2120,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting</t>
+          <t>Palliative Care and End-of-Life Decisions in the UKMLA</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>/news#patient-safety-ukmla-prescribing-errors</t>
+          <t>/news#palliative-care-ukmla-revision</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2134,37 +2134,41 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Cardiology High-Yield Topics for the UKMLA AKT; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Understanding the Foundation Programme: What Awaits After the UKMLA; Good Medical Practice and the UKMLA: What the GMC Expects; How to Read an AKT Stem: Avoiding Common Traps; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Palliative Care and End-of-Life Decisions in the UKMLA; Social Determinants of Health in the UKMLA: Person-Centred Care; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA Results: How to Interpret Your Feedback Report</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>AKT Exam Pattern; CPSA Exam Pattern; Preparation; MLA Content Map / Syllabus; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Good Medical Practice and the UKMLA: What the GMC Expects; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Psychiatry Communication Stations: Handling Difficult Conversations; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know</t>
+          <t>Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Professional Practice &amp; Safety</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr"/>
+          <t>Clinical Systems Revision</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>MLA Content Map / Syllabus</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>PLAB 2 Preparation: How to Excel in the Clinical Assessment</t>
+          <t>Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>/news#plab-2-preparation-guide</t>
+          <t>/news#patient-safety-ukmla-prescribing-errors</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2173,41 +2177,37 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Resits: Rules, Limits, and How to Bounce Back</t>
+          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Cardiology High-Yield Topics for the UKMLA AKT; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Understanding the Foundation Programme: What Awaits After the UKMLA; Good Medical Practice and the UKMLA: What the GMC Expects; How to Read an AKT Stem: Avoiding Common Traps; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Palliative Care and End-of-Life Decisions in the UKMLA; Social Determinants of Health in the UKMLA: Person-Centred Care; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>Appeals and Resits; Preparation; Registration Guide; Results and Scoring; MLA Content Map / Syllabus; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Good Medical Practice and the UKMLA: What the GMC Expects; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; The Role of Mock Exams in UKMLA Preparation; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Psychiatry Communication Stations: Handling Difficult Conversations; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Time Management in the UKMLA AKT: Strategies That Work; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA Results: How to Interpret Your Feedback Report</t>
+          <t>AKT Exam Pattern; CPSA Exam Pattern; Preparation; MLA Content Map / Syllabus; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Good Medical Practice and the UKMLA: What the GMC Expects; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Psychiatry Communication Stations: Handling Difficult Conversations; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Core UKMLA Overview</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>UKMLA vs PLAB</t>
-        </is>
-      </c>
+          <t>Professional Practice &amp; Safety</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Psychiatry Communication Stations: Handling Difficult Conversations</t>
+          <t>PLAB 2 Preparation: How to Excel in the Clinical Assessment</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>/news#psychiatry-communication-cpsa-stations</t>
+          <t>/news#plab-2-preparation-guide</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2216,41 +2216,41 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; Group Study vs Solo Study for the UKMLA: What Works Best?; How to Read an AKT Stem: Avoiding Common Traps; Mental Health Presentations in the UKMLA: What to Revise; The Role of Mock Exams in UKMLA Preparation; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; PLAB 2 Preparation: How to Excel in the Clinical Assessment; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report</t>
+          <t>How to Become a Doctor in the UK from India: The Complete UKMLA Route; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA Resits: Rules, Limits, and How to Bounce Back</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>AKT Exam Pattern; CPSA Exam Pattern; Preparation; MLA Content Map / Syllabus; Cardiology High-Yield Topics for the UKMLA AKT; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Mental Health Presentations in the UKMLA: What to Revise; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Safeguarding Adults and Children: A UKMLA Revision Guide; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know</t>
+          <t>Appeals and Resits; Preparation; Registration Guide; Results and Scoring; MLA Content Map / Syllabus; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Good Medical Practice and the UKMLA: What the GMC Expects; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; The Role of Mock Exams in UKMLA Preparation; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Psychiatry Communication Stations: Handling Difficult Conversations; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Time Management in the UKMLA AKT: Strategies That Work; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA Results: How to Interpret Your Feedback Report</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Exam Format</t>
+          <t>Core UKMLA Overview</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>CPSA Exam Pattern</t>
+          <t>UKMLA vs PLAB</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Radiology and Imaging Interpretation in the AKT</t>
+          <t>Psychiatry Communication Stations: Handling Difficult Conversations</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>/news#radiology-imaging-akt-ukmla</t>
+          <t>/news#psychiatry-communication-cpsa-stations</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2262,38 +2262,38 @@
         <v>16</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Clinical Examination Stations in the CPSA: A Practical Guide; Emergency Medicine and Acute Presentations in the UKMLA; Gastroenterology and Hepatology in the UKMLA AKT; How to Read an AKT Stem: Avoiding Common Traps; MLA Content Map: The Blueprint Behind Every UKMLA Question; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; Time Management in the UKMLA AKT: Strategies That Work; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work</t>
+          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; Group Study vs Solo Study for the UKMLA: What Works Best?; How to Read an AKT Stem: Avoiding Common Traps; Mental Health Presentations in the UKMLA: What to Revise; The Role of Mock Exams in UKMLA Preparation; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; PLAB 2 Preparation: How to Excel in the Clinical Assessment; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Results: How to Interpret Your Feedback Report</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>AKT Exam Pattern; Preparation; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; UKMLA AKT: Format, Question Types, and How to Prepare</t>
+          <t>AKT Exam Pattern; CPSA Exam Pattern; Preparation; MLA Content Map / Syllabus; Cardiology High-Yield Topics for the UKMLA AKT; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Mental Health Presentations in the UKMLA: What to Revise; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Safeguarding Adults and Children: A UKMLA Revision Guide; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Clinical Systems Revision</t>
+          <t>Exam Format</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>MLA Content Map / Syllabus</t>
+          <t>CPSA Exam Pattern</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Respiratory Medicine for the UKMLA: What to Focus On</t>
+          <t>Radiology and Imaging Interpretation in the AKT</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>/news#respiratory-medicine-ukmla-revision</t>
+          <t>/news#radiology-imaging-akt-ukmla</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -2302,19 +2302,19 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Blood Tests and Investigations in the AKT: Data Interpretation Guide; Clinical Examination Stations in the CPSA: A Practical Guide; Emergency Medicine and Acute Presentations in the UKMLA; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Group Study vs Solo Study for the UKMLA: What Works Best?; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Nephrology in the UKMLA: AKI, CKD, and Electrolyte Disorders; Neurology in the UKMLA: High-Yield Topics and Revision Tips; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Palliative Care and End-of-Life Decisions in the UKMLA; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Radiology and Imaging Interpretation in the AKT; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Social Determinants of Health in the UKMLA: Person-Centred Care; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work</t>
+          <t>Clinical Examination Stations in the CPSA: A Practical Guide; Emergency Medicine and Acute Presentations in the UKMLA; Gastroenterology and Hepatology in the UKMLA AKT; How to Read an AKT Stem: Avoiding Common Traps; MLA Content Map: The Blueprint Behind Every UKMLA Question; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; Time Management in the UKMLA AKT: Strategies That Work; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>AKT Exam Pattern; CPSA Exam Pattern; Preparation; MLA Content Map / Syllabus; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Radiology and Imaging Interpretation in the AKT; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know</t>
+          <t>AKT Exam Pattern; Preparation; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; UKMLA AKT: Format, Question Types, and How to Prepare</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2331,12 +2331,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity</t>
+          <t>Respiratory Medicine for the UKMLA: What to Focus On</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>/news#rheumatology-ukmla-revision</t>
+          <t>/news#respiratory-medicine-ukmla-revision</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -2345,19 +2345,19 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>8</v>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Graduate-Entry Medical Students: What Is Different?</t>
+          <t>Blood Tests and Investigations in the AKT: Data Interpretation Guide; Clinical Examination Stations in the CPSA: A Practical Guide; Emergency Medicine and Acute Presentations in the UKMLA; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Group Study vs Solo Study for the UKMLA: What Works Best?; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Nephrology in the UKMLA: AKI, CKD, and Electrolyte Disorders; Neurology in the UKMLA: High-Yield Topics and Revision Tips; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Palliative Care and End-of-Life Decisions in the UKMLA; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Radiology and Imaging Interpretation in the AKT; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Social Determinants of Health in the UKMLA: Person-Centred Care; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>Cardiology High-Yield Topics for the UKMLA AKT; Gastroenterology and Hepatology in the UKMLA AKT; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Respiratory Medicine for the UKMLA: What to Focus On</t>
+          <t>AKT Exam Pattern; CPSA Exam Pattern; Preparation; MLA Content Map / Syllabus; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Radiology and Imaging Interpretation in the AKT; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2374,12 +2374,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Safeguarding Adults and Children: A UKMLA Revision Guide</t>
+          <t>Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>/news#safeguarding-ukmla-revision</t>
+          <t>/news#rheumatology-ukmla-revision</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2391,34 +2391,38 @@
         <v>7</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>How to Read an AKT Stem: Avoiding Common Traps; MLA Content Map: The Blueprint Behind Every UKMLA Question; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Psychiatry Communication Stations: Handling Difficult Conversations; Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA Results: How to Interpret Your Feedback Report</t>
+          <t>Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>AKT Exam Pattern; CPSA Exam Pattern; Preparation; MLA Content Map / Syllabus; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; NICE Guidelines and the AKT: What You Actually Need to Know; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide</t>
+          <t>Cardiology High-Yield Topics for the UKMLA AKT; Gastroenterology and Hepatology in the UKMLA AKT; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Respiratory Medicine for the UKMLA: What to Focus On</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Professional Practice &amp; Safety</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr"/>
+          <t>Clinical Systems Revision</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>MLA Content Map / Syllabus</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Social Determinants of Health in the UKMLA: Person-Centred Care</t>
+          <t>Safeguarding Adults and Children: A UKMLA Revision Guide</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>/news#social-determinants-health-ukmla</t>
+          <t>/news#safeguarding-ukmla-revision</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2427,41 +2431,37 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>MLA Content Map: The Blueprint Behind Every UKMLA Question; Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA Fees: The Complete 2026 Cost Breakdown; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>How to Read an AKT Stem: Avoiding Common Traps; MLA Content Map: The Blueprint Behind Every UKMLA Question; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Psychiatry Communication Stations: Handling Difficult Conversations; Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA Results: How to Interpret Your Feedback Report</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>Appeals and Resits; AKT Exam Pattern; Cardiology High-Yield Topics for the UKMLA AKT; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Respiratory Medicine for the UKMLA: What to Focus On</t>
+          <t>AKT Exam Pattern; CPSA Exam Pattern; Preparation; MLA Content Map / Syllabus; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; NICE Guidelines and the AKT: What You Actually Need to Know; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Clinical Systems Revision</t>
-        </is>
-      </c>
-      <c r="I49" s="2" t="inlineStr">
-        <is>
-          <t>MLA Content Map / Syllabus</t>
-        </is>
-      </c>
+          <t>Professional Practice &amp; Safety</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know</t>
+          <t>Social Determinants of Health in the UKMLA: Person-Centred Care</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>/news#surgical-presentations-ukmla-revision</t>
+          <t>/news#social-determinants-health-ukmla</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2470,19 +2470,19 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Emergency Medicine and Acute Presentations in the UKMLA; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; Gastroenterology and Hepatology in the UKMLA AKT; Good Medical Practice and the UKMLA: What the GMC Expects; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; How to Read an AKT Stem: Avoiding Common Traps; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; MLA Content Map: The Blueprint Behind Every UKMLA Question; Nephrology in the UKMLA: AKI, CKD, and Electrolyte Disorders; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Palliative Care and End-of-Life Decisions in the UKMLA; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Three Months to the UKMLA AKT: A Final Preparation Countdown; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report</t>
+          <t>MLA Content Map: The Blueprint Behind Every UKMLA Question; Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>Preparation; MLA Content Map / Syllabus; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On</t>
+          <t>Appeals and Resits; AKT Exam Pattern; Cardiology High-Yield Topics for the UKMLA AKT; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Respiratory Medicine for the UKMLA: What to Focus On</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2499,12 +2499,12 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Three Months to the UKMLA AKT: A Final Preparation Countdown</t>
+          <t>Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>/news#three-months-ukmla-akt-countdown</t>
+          <t>/news#surgical-presentations-ukmla-revision</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -2513,41 +2513,41 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>Mental Health Presentations in the UKMLA: What to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
+          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Emergency Medicine and Acute Presentations in the UKMLA; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; Gastroenterology and Hepatology in the UKMLA AKT; Good Medical Practice and the UKMLA: What the GMC Expects; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; How to Read an AKT Stem: Avoiding Common Traps; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; MLA Content Map: The Blueprint Behind Every UKMLA Question; Nephrology in the UKMLA: AKI, CKD, and Electrolyte Disorders; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Palliative Care and End-of-Life Decisions in the UKMLA; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Three Months to the UKMLA AKT: A Final Preparation Countdown; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>AKT Exam Pattern; CPSA Exam Pattern; Preparation; MLA Content Map / Syllabus; Cardiology High-Yield Topics for the UKMLA AKT; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Gastroenterology and Hepatology in the UKMLA AKT; Good Medical Practice and the UKMLA: What the GMC Expects; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; How to Read an AKT Stem: Avoiding Common Traps; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Nephrology in the UKMLA: AKI, CKD, and Electrolyte Disorders; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Palliative Care and End-of-Life Decisions in the UKMLA; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Safeguarding Adults and Children: A UKMLA Revision Guide; Social Determinants of Health in the UKMLA: Person-Centred Care; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; How UK Medical Schools Implement the UKMLA: An Overview</t>
+          <t>Preparation; MLA Content Map / Syllabus; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Exam Preparation</t>
+          <t>Clinical Systems Revision</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>Preparation</t>
+          <t>MLA Content Map / Syllabus</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Time Management in the UKMLA AKT: Strategies That Work</t>
+          <t>Three Months to the UKMLA AKT: A Final Preparation Countdown</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>/news#time-management-akt-ukmla</t>
+          <t>/news#three-months-ukmla-akt-countdown</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -2556,19 +2556,19 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Blood Tests and Investigations in the AKT: Data Interpretation Guide; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Group Study vs Solo Study for the UKMLA: What Works Best?; PLAB 2 Preparation: How to Excel in the Clinical Assessment; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA Results: How to Interpret Your Feedback Report</t>
+          <t>Mental Health Presentations in the UKMLA: What to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>Appeals and Resits; AKT Exam Pattern; Preparation; MLA Content Map / Syllabus; UKMLA vs PLAB; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Gastroenterology and Hepatology in the UKMLA AKT; How to Read an AKT Stem: Avoiding Common Traps; The Role of Mock Exams in UKMLA Preparation; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
+          <t>AKT Exam Pattern; CPSA Exam Pattern; Preparation; MLA Content Map / Syllabus; Cardiology High-Yield Topics for the UKMLA AKT; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Gastroenterology and Hepatology in the UKMLA AKT; Good Medical Practice and the UKMLA: What the GMC Expects; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; How to Read an AKT Stem: Avoiding Common Traps; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Nephrology in the UKMLA: AKI, CKD, and Electrolyte Disorders; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Palliative Care and End-of-Life Decisions in the UKMLA; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Safeguarding Adults and Children: A UKMLA Revision Guide; Social Determinants of Health in the UKMLA: Person-Centred Care; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; How UK Medical Schools Implement the UKMLA: An Overview</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -2585,12 +2585,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>How UK Medical Schools Implement the UKMLA: An Overview</t>
+          <t>Time Management in the UKMLA AKT: Strategies That Work</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>/news#uk-medical-schools-ukmla-implementation</t>
+          <t>/news#time-management-akt-ukmla</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2599,41 +2599,41 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Clinical Examination Stations in the CPSA: A Practical Guide; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; Group Study vs Solo Study for the UKMLA: What Works Best?; How to Read an AKT Stem: Avoiding Common Traps; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; Mental Health Presentations in the UKMLA: What to Revise; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>Blood Tests and Investigations in the AKT: Data Interpretation Guide; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Group Study vs Solo Study for the UKMLA: What Works Best?; PLAB 2 Preparation: How to Excel in the Clinical Assessment; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA Results: How to Interpret Your Feedback Report</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>AKT Exam Pattern; CPSA Exam Pattern; Official Resources; Preparation; Registration Guide; Results and Scoring; MLA Content Map / Syllabus; UKMLA vs PLAB; What Is the UKMLA?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; How to Read an AKT Stem: Avoiding Common Traps; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Time Management in the UKMLA AKT: Strategies That Work; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
+          <t>Appeals and Resits; AKT Exam Pattern; Preparation; MLA Content Map / Syllabus; UKMLA vs PLAB; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Gastroenterology and Hepatology in the UKMLA AKT; How to Read an AKT Stem: Avoiding Common Traps; The Role of Mock Exams in UKMLA Preparation; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Core UKMLA Overview</t>
+          <t>Exam Preparation</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>What Is the UKMLA?</t>
+          <t>Preparation</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>UKMLA AKT: Format, Question Types, and How to Prepare</t>
+          <t>How UK Medical Schools Implement the UKMLA: An Overview</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>/news#ukmla-akt-format-preparation</t>
+          <t>/news#uk-medical-schools-ukmla-implementation</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -2642,41 +2642,41 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Radiology and Imaging Interpretation in the AKT; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA for Graduate-Entry Medical Students: What Is Different?; How to Write UKMLA Revision Notes That Actually Work</t>
+          <t>What Is an Angoff Standard Setting and Why Does It Matter?; Clinical Examination Stations in the CPSA: A Practical Guide; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; Group Study vs Solo Study for the UKMLA: What Works Best?; How to Become a Doctor in the UK from India: The Complete UKMLA Route; How to Read an AKT Stem: Avoiding Common Traps; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; Mental Health Presentations in the UKMLA: What to Revise; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs PLAB: What Is the Difference?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>Appeals and Resits; AKT Exam Pattern; CPSA Exam Pattern; Official Resources; Preparation; Registration Guide; Results and Scoring; MLA Content Map / Syllabus; UKMLA vs PLAB; What Is the UKMLA?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; Gastroenterology and Hepatology in the UKMLA AKT; Good Medical Practice and the UKMLA: What the GMC Expects; How to Read an AKT Stem: Avoiding Common Traps; Neurology in the UKMLA: High-Yield Topics and Revision Tips; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Safeguarding Adults and Children: A UKMLA Revision Guide; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Results: How to Interpret Your Feedback Report; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>AKT Exam Pattern; CPSA Exam Pattern; Official Resources; Preparation; Registration Guide; Results and Scoring; MLA Content Map / Syllabus; UKMLA vs PLAB; What Is the UKMLA?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; How to Read an AKT Stem: Avoiding Common Traps; Respiratory Medicine for the UKMLA: What to Focus On; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Time Management in the UKMLA AKT: Strategies That Work; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Exam Format</t>
+          <t>Core UKMLA Overview</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>AKT Exam Pattern</t>
+          <t>What Is the UKMLA?</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>UKMLA CPSA: What the Clinical Exam Really Tests</t>
+          <t>UKMLA AKT: Format, Question Types, and How to Prepare</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>/news#ukmla-cpsa-what-it-tests</t>
+          <t>/news#ukmla-akt-format-preparation</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -2685,19 +2685,19 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Mental Health Presentations in the UKMLA: What to Revise; Neurology in the UKMLA: High-Yield Topics and Revision Tips; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>How to Become a Doctor in the UK from India: The Complete UKMLA Route; MLA Content Map: The Blueprint Behind Every UKMLA Question; The Role of Mock Exams in UKMLA Preparation; Radiology and Imaging Interpretation in the AKT; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; CPSA Exam Pattern; Preparation; Results and Scoring; MLA Content Map / Syllabus; UKMLA vs PLAB; What Is the UKMLA?; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Psychiatry Communication Stations: Handling Difficult Conversations; Respiratory Medicine for the UKMLA: What to Focus On; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report</t>
+          <t>Appeals and Resits; AKT Exam Pattern; CPSA Exam Pattern; Official Resources; Preparation; Registration Guide; Results and Scoring; MLA Content Map / Syllabus; UKMLA vs PLAB; What Is the UKMLA?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; Gastroenterology and Hepatology in the UKMLA AKT; Good Medical Practice and the UKMLA: What the GMC Expects; How to Read an AKT Stem: Avoiding Common Traps; Neurology in the UKMLA: High-Yield Topics and Revision Tips; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Safeguarding Adults and Children: A UKMLA Revision Guide; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Results: How to Interpret Your Feedback Report; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -2707,19 +2707,19 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>CPSA Exam Pattern</t>
+          <t>AKT Exam Pattern</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>UKMLA Eligibility: Who Can Sit the Exam?</t>
+          <t>UKMLA CPSA: What the Clinical Exam Really Tests</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>/news#ukmla-eligibility-who-can-sit</t>
+          <t>/news#ukmla-cpsa-what-it-tests</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2728,41 +2728,41 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>How to Register for PLAB 1: A Step-by-Step Guide for IMGs; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
+          <t>Mental Health Presentations in the UKMLA: What to Revise; Neurology in the UKMLA: High-Yield Topics and Revision Tips; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; CPSA Exam Pattern; Registration Guide; What Is the UKMLA?; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
+          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; CPSA Exam Pattern; Preparation; Results and Scoring; MLA Content Map / Syllabus; UKMLA vs PLAB; What Is the UKMLA?; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Neurology in the UKMLA: High-Yield Topics and Revision Tips; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Psychiatry Communication Stations: Handling Difficult Conversations; Respiratory Medicine for the UKMLA: What to Focus On; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Registration &amp; Eligibility</t>
+          <t>Exam Format</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>Eligibility</t>
+          <t>CPSA Exam Pattern</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>UKMLA Fees: The Complete 2026 Cost Breakdown</t>
+          <t>UKMLA Eligibility: Who Can Sit the Exam?</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>/news#ukmla-fees-explained</t>
+          <t>/news#ukmla-eligibility-who-can-sit</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -2771,19 +2771,19 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report</t>
+          <t>How to Become a Doctor in the UK from India: The Complete UKMLA Route; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; CPSA Exam Pattern; Fees; Key Dates; Official Resources; Preparation; Registration Guide; Results and Scoring; MLA Content Map / Syllabus; UKMLA vs PLAB; Social Determinants of Health in the UKMLA: Person-Centred Care; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
+          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; CPSA Exam Pattern; Registration Guide; What Is the UKMLA?; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -2793,19 +2793,19 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>Fees</t>
+          <t>Eligibility</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>UKMLA for Graduate-Entry Medical Students: What Is Different?</t>
+          <t>UKMLA Fees: The Complete 2026 Cost Breakdown</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>/news#ukmla-graduate-entry-medical-students</t>
+          <t>/news#ukmla-fees-explained</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -2814,41 +2814,41 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Key Dates and Sitting Schedule: What to Know</t>
+          <t>How to Become a Doctor in the UK from India: The Complete UKMLA Route; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>Appeals and Resits; Eligibility; Official Resources; Preparation; Results and Scoring; MLA Content Map / Syllabus; What Is the UKMLA?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Understanding the Foundation Programme: What Awaits After the UKMLA; Good Medical Practice and the UKMLA: What the GMC Expects; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; How to Read an AKT Stem: Avoiding Common Traps; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; Neurology in the UKMLA: High-Yield Topics and Revision Tips; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests</t>
+          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; CPSA Exam Pattern; Fees; Key Dates; Official Resources; Preparation; Registration Guide; Results and Scoring; MLA Content Map / Syllabus; UKMLA vs PLAB; Social Determinants of Health in the UKMLA: Person-Centred Care; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Core UKMLA Overview</t>
+          <t>Registration &amp; Eligibility</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>Eligibility</t>
+          <t>Fees</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>UKMLA Key Dates and Sitting Schedule: What to Know</t>
+          <t>UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>/news#ukmla-key-dates-sitting-schedule</t>
+          <t>/news#ukmla-fees-for-img-2026</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -2857,19 +2857,19 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Group Study vs Solo Study for the UKMLA: What Works Best?; How to Register for PLAB 1: A Step-by-Step Guide for IMGs</t>
+          <t>How to Become a Doctor in the UK from India: The Complete UKMLA Route; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>Appeals and Resits; Eligibility; Fees; Official Resources; Preparation; Results and Scoring; UKMLA vs PLAB; Understanding the Foundation Programme: What Awaits After the UKMLA; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Results: How to Interpret Your Feedback Report</t>
+          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; CPSA Exam Pattern; Fees; Key Dates; Official Resources; Preparation; Registration Guide; MLA Content Map / Syllabus; UKMLA vs PLAB; How to Become a Doctor in the UK from India: The Complete UKMLA Route; The Role of Mock Exams in UKMLA Preparation; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -2879,19 +2879,19 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>Key Dates</t>
+          <t>Fees</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
+          <t>UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>/news#ukmla-preparation-for-imgs</t>
+          <t>/news#ukmla-for-nigerian-doctors</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -2900,41 +2900,41 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA vs PLAB: What Is the Difference?; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>Appeals and Resits; Eligibility; Fees; Key Dates; Official Resources; Preparation; Registration Guide; MLA Content Map / Syllabus; UKMLA vs PLAB; Clinical Examination Stations in the CPSA: A Practical Guide; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; How to Read an AKT Stem: Avoiding Common Traps; Mental Health Presentations in the UKMLA: What to Revise; NICE Guidelines and the AKT: What You Actually Need to Know; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown</t>
+          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; CPSA Exam Pattern; Fees; Key Dates; Official Resources; Preparation; Registration Guide; MLA Content Map / Syllabus; UKMLA vs PLAB; Emergency Medicine and Acute Presentations in the UKMLA; Understanding the Foundation Programme: What Awaits After the UKMLA; How to Become a Doctor in the UK from India: The Complete UKMLA Route; MLA Content Map: The Blueprint Behind Every UKMLA Question; NICE Guidelines and the AKT: What You Actually Need to Know; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Psychiatry Communication Stations: Handling Difficult Conversations; Social Determinants of Health in the UKMLA: Person-Centred Care; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Core UKMLA Overview</t>
+          <t>IMG Country Routes &amp; Global Comparisons</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>UKMLA vs PLAB</t>
+          <t>Eligibility</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>UKMLA Resits: Rules, Limits, and How to Bounce Back</t>
+          <t>UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>/news#ukmla-resits-rules-limits</t>
+          <t>/news#ukmla-for-pakistani-doctors</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -2946,38 +2946,38 @@
         <v>2</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>PLAB 2 Preparation: How to Excel in the Clinical Assessment; UKMLA Results: How to Interpret Your Feedback Report</t>
+          <t>UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>Appeals and Resits; Fees; Preparation; Results and Scoring; UKMLA vs PLAB; The Role of Mock Exams in UKMLA Preparation; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work</t>
+          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; CPSA Exam Pattern; Fees; Key Dates; Official Resources; Preparation; Registration Guide; Results and Scoring; MLA Content Map / Syllabus; UKMLA vs PLAB; What Is the UKMLA?; Cardiology High-Yield Topics for the UKMLA AKT; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Emergency Medicine and Acute Presentations in the UKMLA; Understanding the Foundation Programme: What Awaits After the UKMLA; How to Become a Doctor in the UK from India: The Complete UKMLA Route; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; The Role of Mock Exams in UKMLA Preparation; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Three Months to the UKMLA AKT: A Final Preparation Countdown; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Resits: Rules, Limits, and How to Bounce Back</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Registration &amp; Eligibility</t>
+          <t>IMG Country Routes &amp; Global Comparisons</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Appeals and Resits</t>
+          <t>Eligibility</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>UKMLA Results: How to Interpret Your Feedback Report</t>
+          <t>UKMLA for Graduate-Entry Medical Students: What Is Different?</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>/news#ukmla-results-feedback-report</t>
+          <t>/news#ukmla-graduate-entry-medical-students</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -2986,41 +2986,41 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>31</v>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>PLAB 2 Preparation: How to Excel in the Clinical Assessment; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Resits: Rules, Limits, and How to Bounce Back</t>
+          <t>How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Key Dates and Sitting Schedule: What to Know</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; Official Resources; Preparation; Results and Scoring; MLA Content Map / Syllabus; UKMLA vs PLAB; What Is an Angoff Standard Setting and Why Does It Matter?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Understanding the Foundation Programme: What Awaits After the UKMLA; Good Medical Practice and the UKMLA: What the GMC Expects; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; How to Read an AKT Stem: Avoiding Common Traps; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Palliative Care and End-of-Life Decisions in the UKMLA; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Safeguarding Adults and Children: A UKMLA Revision Guide; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Resits: Rules, Limits, and How to Bounce Back</t>
+          <t>Appeals and Resits; Eligibility; Official Resources; Preparation; Results and Scoring; MLA Content Map / Syllabus; What Is the UKMLA?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Understanding the Foundation Programme: What Awaits After the UKMLA; Good Medical Practice and the UKMLA: What the GMC Expects; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; How to Read an AKT Stem: Avoiding Common Traps; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Mental Health Presentations in the UKMLA: What to Revise; Neurology in the UKMLA: High-Yield Topics and Revision Tips; NICE Guidelines and the AKT: What You Actually Need to Know; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Results &amp; Scoring</t>
+          <t>Core UKMLA Overview</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Results and Scoring</t>
+          <t>Eligibility</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>How to Write UKMLA Revision Notes That Actually Work</t>
+          <t>UKMLA Key Dates and Sitting Schedule: What to Know</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>/news#ukmla-revision-notes-strategy</t>
+          <t>/news#ukmla-key-dates-sitting-schedule</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -3029,41 +3029,41 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Group Study vs Solo Study for the UKMLA: What Works Best?; UKMLA Resits: Rules, Limits, and How to Bounce Back</t>
+          <t>Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; Group Study vs Solo Study for the UKMLA: What Works Best?; How to Become a Doctor in the UK from India: The Complete UKMLA Route; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>AKT Exam Pattern; CPSA Exam Pattern; Official Resources; Preparation; MLA Content Map / Syllabus; What Is the UKMLA?; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Good Medical Practice and the UKMLA: What the GMC Expects; Group Study vs Solo Study for the UKMLA: What Works Best?; Neurology in the UKMLA: High-Yield Topics and Revision Tips; NICE Guidelines and the AKT: What You Actually Need to Know; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare</t>
+          <t>Appeals and Resits; Eligibility; Fees; Official Resources; Preparation; Results and Scoring; UKMLA vs PLAB; Understanding the Foundation Programme: What Awaits After the UKMLA; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA for Graduate-Entry Medical Students: What Is Different?; UKMLA Results: How to Interpret Your Feedback Report</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Exam Preparation</t>
+          <t>Registration &amp; Eligibility</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Preparation</t>
+          <t>Key Dates</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>UKMLA vs PLAB: What Is the Difference?</t>
+          <t>UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>/news#ukmla-vs-plab-difference</t>
+          <t>/news#ukmla-preparation-for-imgs</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -3072,19 +3072,19 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>MLA Content Map: The Blueprint Behind Every UKMLA Question; What Is the UKMLA? A Complete Beginner's Guide</t>
+          <t>How to Become a Doctor in the UK from India: The Complete UKMLA Route; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Resits: Rules, Limits, and How to Bounce Back; UKMLA vs PLAB: What Is the Difference?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?; What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; CPSA Exam Pattern; Fees; Official Resources; Registration Guide; Results and Scoring; MLA Content Map / Syllabus; UKMLA vs PLAB; What Is the UKMLA?; Understanding the Foundation Programme: What Awaits After the UKMLA; How to Read an AKT Stem: Avoiding Common Traps; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; The Role of Mock Exams in UKMLA Preparation; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
+          <t>Appeals and Resits; Eligibility; Fees; Key Dates; Official Resources; Preparation; Registration Guide; MLA Content Map / Syllabus; UKMLA vs PLAB; Clinical Examination Stations in the CPSA: A Practical Guide; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; How to Read an AKT Stem: Avoiding Common Traps; Mental Health Presentations in the UKMLA: What to Revise; NICE Guidelines and the AKT: What You Actually Need to Know; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Fees: The Complete 2026 Cost Breakdown</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3101,48 +3101,349 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
+          <t>UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>/news#ukmla-question-bank-and-mock-tests</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Blog Post</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E65" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>How to Become a Doctor in the UK from India: The Complete UKMLA Route; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>Eligibility; AKT Exam Pattern; Fees; Official Resources; Preparation; Results and Scoring; MLA Content Map / Syllabus; Cardiology High-Yield Topics for the UKMLA AKT; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide; How to Become a Doctor in the UK from India: The Complete UKMLA Route; How to Read an AKT Stem: Avoiding Common Traps; The Role of Mock Exams in UKMLA Preparation; Ophthalmology and ENT in the UKMLA: What Foundation Doctors Need to Know; Psychiatry Communication Stations: Handling Difficult Conversations; Respiratory Medicine for the UKMLA: What to Focus On; Rheumatology in the UKMLA: Joints, Inflammation, and Autoimmunity; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Nigerian Doctors: Eligibility, Fees and How to Register with the GMC; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA Preparation for IMG Candidates: A Tailored Guide; How to Write UKMLA Revision Notes That Actually Work; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>IMG Country Routes &amp; Global Comparisons</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Preparation</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>UKMLA Resits: Rules, Limits, and How to Bounce Back</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>/news#ukmla-resits-rules-limits</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Blog Post</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>PLAB 2 Preparation: How to Excel in the Clinical Assessment; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA for Pakistani Doctors: Eligibility, Fees and the Route to Practising in the UK; UKMLA Results: How to Interpret Your Feedback Report</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>Appeals and Resits; Fees; Preparation; Results and Scoring; UKMLA vs PLAB; The Role of Mock Exams in UKMLA Preparation; PLAB 2 Preparation: How to Excel in the Clinical Assessment; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Results: How to Interpret Your Feedback Report; How to Write UKMLA Revision Notes That Actually Work</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Registration &amp; Eligibility</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>Appeals and Resits</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>UKMLA Results: How to Interpret Your Feedback Report</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>/news#ukmla-results-feedback-report</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Blog Post</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E67" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>PLAB 2 Preparation: How to Excel in the Clinical Assessment; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Key Dates and Sitting Schedule: What to Know; UKMLA Resits: Rules, Limits, and How to Bounce Back</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; Official Resources; Preparation; Results and Scoring; MLA Content Map / Syllabus; UKMLA vs PLAB; What Is an Angoff Standard Setting and Why Does It Matter?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; Disability, Access, and Inclusion in the UKMLA: A Candidate's Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Understanding the Foundation Programme: What Awaits After the UKMLA; Good Medical Practice and the UKMLA: What the GMC Expects; Haematology in the UKMLA: Anaemia, Clotting, and Blood Cancers; How to Read an AKT Stem: Avoiding Common Traps; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Palliative Care and End-of-Life Decisions in the UKMLA; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Psychiatry Communication Stations: Handling Difficult Conversations; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; Safeguarding Adults and Children: A UKMLA Revision Guide; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Time Management in the UKMLA AKT: Strategies That Work; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Fees: The Complete 2026 Cost Breakdown; UKMLA Resits: Rules, Limits, and How to Bounce Back</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>Results &amp; Scoring</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>Results and Scoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>How to Write UKMLA Revision Notes That Actually Work</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>/news#ukmla-revision-notes-strategy</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Blog Post</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>Group Study vs Solo Study for the UKMLA: What Works Best?; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA Resits: Rules, Limits, and How to Bounce Back</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>AKT Exam Pattern; CPSA Exam Pattern; Official Resources; Preparation; MLA Content Map / Syllabus; What Is the UKMLA?; Cardiology High-Yield Topics for the UKMLA AKT; Clinical Examination Stations in the CPSA: A Practical Guide; ECG Interpretation for the UKMLA: The Findings You Must Recognise; Good Medical Practice and the UKMLA: What the GMC Expects; Group Study vs Solo Study for the UKMLA: What Works Best?; Neurology in the UKMLA: High-Yield Topics and Revision Tips; NICE Guidelines and the AKT: What You Actually Need to Know; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Radiology and Imaging Interpretation in the AKT; Respiratory Medicine for the UKMLA: What to Focus On; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Exam Preparation</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>Preparation</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>/news#ukmla-vs-neet-pg</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Blog Post</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>How to Become a Doctor in the UK from India: The Complete UKMLA Route; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; CPSA Exam Pattern; Fees; Preparation; Registration Guide; MLA Content Map / Syllabus; UKMLA vs PLAB; What Is the UKMLA?; Blood Tests and Investigations in the AKT: Data Interpretation Guide; Clinical Examination Stations in the CPSA: A Practical Guide; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Understanding the Foundation Programme: What Awaits After the UKMLA; How to Become a Doctor in the UK from India: The Complete UKMLA Route; MLA Content Map: The Blueprint Behind Every UKMLA Question; Obstetrics and Gynaecology in the UKMLA: Key Topics to Revise; Paediatrics in the AKT and CPSA: A Focused Revision Guide; Radiology and Imaging Interpretation in the AKT; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA vs PLAB: What Is the Difference?; UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>IMG Country Routes &amp; Global Comparisons</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>UKMLA vs PLAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>UKMLA vs PLAB: What Is the Difference?</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>/news#ukmla-vs-plab-difference</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Blog Post</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>MLA Content Map: The Blueprint Behind Every UKMLA Question; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?; What Is the UKMLA? A Complete Beginner's Guide</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>Appeals and Resits; Eligibility; AKT Exam Pattern; CPSA Exam Pattern; Fees; Official Resources; Registration Guide; Results and Scoring; MLA Content Map / Syllabus; UKMLA vs PLAB; What Is the UKMLA?; Understanding the Foundation Programme: What Awaits After the UKMLA; How to Read an AKT Stem: Avoiding Common Traps; How to Register for PLAB 1: A Step-by-Step Guide for IMGs; The Role of Mock Exams in UKMLA Preparation; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA Preparation for IMG Candidates: A Tailored Guide</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Core UKMLA Overview</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>UKMLA vs PLAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>UKMLA vs USMLE: Which Exam Is Easier, Cheaper and Better for Your Career?</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>/news#ukmla-vs-usmle-comparison</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Blog Post</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E71" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>How to Become a Doctor in the UK from India: The Complete UKMLA Route; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources; UKMLA vs NEET PG: Which Path Should Indian Medical Graduates Choose?</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>Appeals and Resits; AKT Exam Pattern; CPSA Exam Pattern; Fees; Preparation; Registration Guide; Results and Scoring; MLA Content Map / Syllabus; UKMLA vs PLAB; What Is the UKMLA?; What Is an Angoff Standard Setting and Why Does It Matter?; Clinical Examination Stations in the CPSA: A Practical Guide; Dermatology in the UKMLA: Rashes, Lesions, and What to Know; Understanding the Foundation Programme: What Awaits After the UKMLA; How to Become a Doctor in the UK from India: The Complete UKMLA Route; Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More; Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know; Three Months to the UKMLA AKT: A Final Preparation Countdown; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA AKT: Format, Question Types, and How to Prepare; UKMLA Eligibility: Who Can Sit the Exam?; UKMLA Exam Fees for International Medical Graduates: 2026 Cost Guide; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA Question Bank and Mock Tests: The Complete Guide to Practice Resources</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>IMG Country Routes &amp; Global Comparisons</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>UKMLA vs PLAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
           <t>What Is the UKMLA? A Complete Beginner's Guide</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>/news#what-is-ukmla-complete-guide</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>Blog Post</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="n">
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Blog Post</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E65" s="2" t="n">
+      <c r="E72" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="F65" s="3" t="inlineStr">
+      <c r="F72" s="3" t="inlineStr">
         <is>
           <t>Understanding the Foundation Programme: What Awaits After the UKMLA; UKMLA AKT: Format, Question Types, and How to Prepare</t>
         </is>
       </c>
-      <c r="G65" s="3" t="inlineStr">
+      <c r="G72" s="3" t="inlineStr">
         <is>
           <t>Appeals and Resits; Eligibility; AKT Exam Pattern; CPSA Exam Pattern; Fees; Official Resources; Preparation; Registration Guide; Results and Scoring; MLA Content Map / Syllabus; UKMLA vs PLAB; What Is the UKMLA?; What Is an Angoff Standard Setting and Why Does It Matter?; Clinical Examination Stations in the CPSA: A Practical Guide; Understanding the Foundation Programme: What Awaits After the UKMLA; Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting; Social Determinants of Health in the UKMLA: Person-Centred Care; How UK Medical Schools Implement the UKMLA: An Overview; UKMLA CPSA: What the Clinical Exam Really Tests; UKMLA Preparation for IMG Candidates: A Tailored Guide; UKMLA vs PLAB: What Is the Difference?</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="H72" s="2" t="inlineStr">
         <is>
           <t>Core UKMLA Overview</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr">
+      <c r="I72" s="2" t="inlineStr">
         <is>
           <t>What Is the UKMLA?</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I65"/>
+  <autoFilter ref="A1:I72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3179,7 +3480,7 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>51</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3">
@@ -3199,7 +3500,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>734</v>
+        <v>905</v>
       </c>
     </row>
     <row r="5">
@@ -3209,7 +3510,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>14.4</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="6">
@@ -3260,7 +3561,7 @@
       <c r="A12" s="5" t="inlineStr"/>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know (31 incoming)</t>
+          <t>Surgical Presentations in the UKMLA: What a Foundation Doctor Needs to Know (33 incoming)</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3569,7 @@
       <c r="A13" s="5" t="inlineStr"/>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Respiratory Medicine for the UKMLA: What to Focus On (30 incoming)</t>
+          <t>Respiratory Medicine for the UKMLA: What to Focus On (31 incoming)</t>
         </is>
       </c>
     </row>
@@ -3276,7 +3577,7 @@
       <c r="A14" s="5" t="inlineStr"/>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Paediatrics in the AKT and CPSA: A Focused Revision Guide (27 incoming)</t>
+          <t>How UK Medical Schools Implement the UKMLA: An Overview (30 incoming)</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3585,7 @@
       <c r="A15" s="5" t="inlineStr"/>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More (25 incoming)</t>
+          <t>Paediatrics in the AKT and CPSA: A Focused Revision Guide (28 incoming)</t>
         </is>
       </c>
     </row>
@@ -3292,7 +3593,7 @@
       <c r="A16" s="5" t="inlineStr"/>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Cardiology High-Yield Topics for the UKMLA AKT (24 incoming)</t>
+          <t>Cardiology High-Yield Topics for the UKMLA AKT (26 incoming)</t>
         </is>
       </c>
     </row>
@@ -3300,7 +3601,7 @@
       <c r="A17" s="5" t="inlineStr"/>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting (24 incoming)</t>
+          <t>Infection and Microbiology in the UKMLA: Antibiotic Stewardship and More (26 incoming)</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3609,7 @@
       <c r="A18" s="5" t="inlineStr"/>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>How UK Medical Schools Implement the UKMLA: An Overview (24 incoming)</t>
+          <t>Patient Safety in the UKMLA: Prescribing Errors and Near-Miss Reporting (25 incoming)</t>
         </is>
       </c>
     </row>
@@ -3316,7 +3617,7 @@
       <c r="A19" s="5" t="inlineStr"/>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>ECG Interpretation for the UKMLA: The Findings You Must Recognise (23 incoming)</t>
+          <t>Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide (24 incoming)</t>
         </is>
       </c>
     </row>
@@ -3324,7 +3625,7 @@
       <c r="A20" s="5" t="inlineStr"/>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Endocrinology and Diabetes in the UKMLA: A Targeted Revision Guide (23 incoming)</t>
+          <t>ECG Interpretation for the UKMLA: The Findings You Must Recognise (23 incoming)</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3633,7 @@
       <c r="A21" s="5" t="inlineStr"/>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Neurology in the UKMLA: High-Yield Topics and Revision Tips (16 incoming)</t>
+          <t>Radiology and Imaging Interpretation in the AKT (17 incoming)</t>
         </is>
       </c>
     </row>

</xml_diff>